<commit_message>
adding coe and tower to back and front
</commit_message>
<xml_diff>
--- a/backend/data/output/one_pager_summary.xlsx
+++ b/backend/data/output/one_pager_summary.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="25" uniqueCount="25">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="26" uniqueCount="26">
   <si>
     <t>section_name</t>
   </si>
@@ -58,65 +58,69 @@
     <t>Role_4</t>
   </si>
   <si>
+    <t>Redacted</t>
+  </si>
+  <si>
     <t>CONTROL TOWER</t>
   </si>
   <si>
-    <t>Experienced data engineer focused on building scalable data platforms and analytics solutions, with expertise in **data engineering**, **ETL**, **data quality**, and **data warehousing**. Hands-on with **AWS**, **Snowflake**, **SQL**, **Python**, **Airflow**, **Matillion**, and delivering **Power BI** reporting and SAP PP/MM support for supply chain.</t>
-  </si>
-  <si>
-    <t>Bachelor Degree in Industrial Engineering</t>
-  </si>
-  <si>
-    <t>Banking
-Chemicals
-Energy
-Industrial</t>
-  </si>
-  <si>
-    <t>Senior Data Engineer
-Data Warehouse Analyst
-Platform Software Engineer
-Supply Chain Analyst
-SAP Consultant PP/MM</t>
-  </si>
-  <si>
-    <t>AWS Cloud Practitioner
-Microsoft Power BI
+    <t>Electronic Engineer and Project Manager with experience as Business Product Owner for MES implementations and leading investment projects in productive machinery. Skilled in **project management**, **industrial automation**, **PLC programming**, **MES requirements**, **data analytics** and **quality assurance**. Proven ability to coordinate multidisciplinary teams, manage budgets and deploy IT-manufacturing solutions.</t>
+  </si>
+  <si>
+    <t>Bachelor of Electronic Engineering
+Postgraduate Project Management</t>
+  </si>
+  <si>
+    <t>Automotive
+Industrial
+High Tech
+Software and Platforms</t>
+  </si>
+  <si>
+    <t>Project Management Lead
+Product Owner MES
+Industrial Automation Engineer
+Quality Assurance Analyst
+Data Analytics Practitioner</t>
+  </si>
+  <si>
+    <t>Python
 SQL
-Python
-Snowflake
-Microsoft SSIS
-Matillion
-Airflow
-Azure DP-900</t>
+PLC Programming
+Power BI
+Jira
+MS Project
+AutoCAD
+Data Analytics
+Project Management</t>
   </si>
   <si>
     <t>Spanish C2
 English C1</t>
   </si>
   <si>
-    <t>Software Engineer Platform – Software platforms
-Designed and implemented scalable data models and services on **SAP BTP** using the **CAP** framework to enable structured backend APIs for enterprise applications.
-Developed and maintained backend data services that enforce business logic and ensure **data integrity**, supporting analytics and reporting pipelines.
-Collaborated with platform teams to integrate services with analytics consumers and improve service reliability and observability.</t>
-  </si>
-  <si>
-    <t>Data Engineer, Quality – Financial Services
-Investigated and resolved data quality issues across the **AWS** data lake, performing root cause analysis with **S3**, **Athena**, **EMR**, **DynamoDB**, and **CloudWatch**.
-Implemented and improved integrity rules in **OvalEdge** using **SQL**, reducing recurring data incidents and impacting ~10% of reported issues.
-Produced **Power BI** reports to communicate quality findings and mentored new team members on data workflows and quality controls.</t>
-  </si>
-  <si>
-    <t>Data Engineer – Financial Services
-Built an end-to-end ingestion pipeline from **Qualtrics** into the **AWS** data lake and loaded curated datasets into **Snowflake** using **Python**, **SQL**, and **GitLab**, orchestrated with **Airflow**.
-Transformed raw data into analytics-ready tables in **Snowflake**, resolving ~40% of data quality issues and improving downstream reporting accuracy.
-Developed an **ELT** process in **Matillion** to support Customer Experience stakeholders, optimizing data delivery and traceability.</t>
-  </si>
-  <si>
-    <t>Data Warehouse Analyst – Oil &amp; Gas
-Monitored and analyzed ETL workflows in **SSIS**, performing **SQL** performance analysis to identify pipeline bottlenecks, anomalies, and inefficiencies.
-Delivered a **Power BI** report on data warehouse performance that uncovered optimization opportunities and reduced failures due to package dependencies by 15%.
-Executed data troubleshooting and remediation to improve ETL reliability and support operational analytics.</t>
+    <t>Senior Project Engineering Analyst
+Served as Business Product Owner for implementation of **MES** projects within IT, leading functional requirement definition, end-user and analyst training, and stakeholder alignment across operations and management.
+Managed capital equipment investment projects including planning, schedule control, resource allocation and budget administration using **MS Project** and formal project controls.
+Coordinated multidisciplinary and global IT teams, defined technical specifications and executed **vendor management** for successful integration and deployment of corporate IT solutions.</t>
+  </si>
+  <si>
+    <t>Quality Assurance Intern
+Executed manual, descriptive and functional testing following **Agile** and **Kanban** methodologies, documenting defects and validating fixes to improve software reliability.
+Managed issue tracking and test workflows using **Jira**, supporting regression testing, defect triage and release readiness.
+Prepared and maintained **test documentation** and contributed process improvement suggestions that streamlined QA activities and reporting.</t>
+  </si>
+  <si>
+    <t>Automation &amp; PLC Engineering Intern
+Contributed to implementation projects for **AGV** systems, performing design support, assembly, programming and commissioning to integrate automated vehicles into production lines.
+Developed and programmed control logic using **PLC Programming**, conducted start-up, troubleshooting and preventive maintenance of automation equipment.
+Performed system integration and validation testing, produced technical documentation and supported operational handover to maintenance and operations teams.</t>
+  </si>
+  <si>
+    <t>STEM Instructor &amp; Lecturer
+Designed and delivered programming, robotics and electronics curricula for children (4–15) emphasizing **STEAM**, hands-on projects and computational thinking to foster sustained engagement.
+Led university practical sessions for **Electrical Circuits**, developed lab exercises, graded assessments and mentored teaching assistants to improve student learning outcomes.
+Created instructional materials and applied **active-learning methodologies** to increase practical competency and curiosity-driven problem solving.</t>
   </si>
 </sst>
 </file>
@@ -489,13 +493,16 @@
       <c r="A2" t="s">
         <v>2</v>
       </c>
+      <c r="B2" t="s">
+        <v>14</v>
+      </c>
     </row>
     <row r="3" spans="1:2">
       <c r="A3" t="s">
         <v>3</v>
       </c>
       <c r="B3" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
     </row>
     <row r="4" spans="1:2">
@@ -503,7 +510,7 @@
         <v>4</v>
       </c>
       <c r="B4" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
     </row>
     <row r="5" spans="1:2">
@@ -511,7 +518,7 @@
         <v>5</v>
       </c>
       <c r="B5" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
     </row>
     <row r="6" spans="1:2">
@@ -519,7 +526,7 @@
         <v>6</v>
       </c>
       <c r="B6" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
     </row>
     <row r="7" spans="1:2">
@@ -527,7 +534,7 @@
         <v>7</v>
       </c>
       <c r="B7" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
     </row>
     <row r="8" spans="1:2">
@@ -535,7 +542,7 @@
         <v>8</v>
       </c>
       <c r="B8" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
     </row>
     <row r="9" spans="1:2">
@@ -543,7 +550,7 @@
         <v>9</v>
       </c>
       <c r="B9" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
     </row>
     <row r="10" spans="1:2">
@@ -551,7 +558,7 @@
         <v>10</v>
       </c>
       <c r="B10" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
     </row>
     <row r="11" spans="1:2">
@@ -559,7 +566,7 @@
         <v>11</v>
       </c>
       <c r="B11" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
     </row>
     <row r="12" spans="1:2">
@@ -567,7 +574,7 @@
         <v>12</v>
       </c>
       <c r="B12" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
     </row>
     <row r="13" spans="1:2">
@@ -575,7 +582,7 @@
         <v>13</v>
       </c>
       <c r="B13" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
adding coe and tower back and front
</commit_message>
<xml_diff>
--- a/backend/data/output/one_pager_summary.xlsx
+++ b/backend/data/output/one_pager_summary.xlsx
@@ -58,13 +58,13 @@
     <t>Role_4</t>
   </si>
   <si>
-    <t>Redacted</t>
-  </si>
-  <si>
-    <t>CONTROL TOWER</t>
-  </si>
-  <si>
-    <t>Electronic Engineer and Project Manager with experience as Business Product Owner for MES implementations and leading investment projects in productive machinery. Skilled in **project management**, **industrial automation**, **PLC programming**, **MES requirements**, **data analytics** and **quality assurance**. Proven ability to coordinate multidisciplinary teams, manage budgets and deploy IT-manufacturing solutions.</t>
+    <t>Paula María Fernández</t>
+  </si>
+  <si>
+    <t>Tower 1</t>
+  </si>
+  <si>
+    <t>Electronic engineer and project manager experienced in leading MES and automation initiatives as product owner and coordinating multidisciplinary teams. Skilled in **Python**, **SQL**, **Power BI**, **ETL**, **analytics**, **automation** and PLC programming; strong focus on requirements, delivery and process optimization.</t>
   </si>
   <si>
     <t>Bachelor of Electronic Engineering
@@ -79,20 +79,21 @@
   <si>
     <t>Project Management Lead
 Product Owner MES
-Industrial Automation Engineer
+Automation Systems Engineer
+Data Analytics Specialist
 Quality Assurance Analyst
-Data Analytics Practitioner</t>
-  </si>
-  <si>
-    <t>Python
+PLC Programming Engineer</t>
+  </si>
+  <si>
+    <t>Project Management PMI
+Data Analytics
+Python
 SQL
+Power BI
 PLC Programming
-Power BI
+Agile Kanban
 Jira
-MS Project
-AutoCAD
-Data Analytics
-Project Management</t>
+MS Project</t>
   </si>
   <si>
     <t>Spanish C2
@@ -100,27 +101,28 @@
   </si>
   <si>
     <t>Senior Project Engineering Analyst
-Served as Business Product Owner for implementation of **MES** projects within IT, leading functional requirement definition, end-user and analyst training, and stakeholder alignment across operations and management.
-Managed capital equipment investment projects including planning, schedule control, resource allocation and budget administration using **MS Project** and formal project controls.
-Coordinated multidisciplinary and global IT teams, defined technical specifications and executed **vendor management** for successful integration and deployment of corporate IT solutions.</t>
+Acted as business product owner for implementation of **MES** projects within **IT**, defining functional requirements and delivering end-user and analyst **training**.
+Managed investment projects for production machinery, overseeing **project management** activities including planning, execution, monitoring and change control.
+Coordinated **multidisciplinary teams**, defined technical specifications and led **vendor management** to ensure on-time delivery of hardware and software components.
+Controlled schedules, resource allocation and budgets using **MS Project**, driving requirements prioritization and alignment with global IT initiatives.</t>
+  </si>
+  <si>
+    <t>Senior Programming and Robotics Instructor
+Designed and delivered age-appropriate curricula to teach **programming**, **robotics** and **electronics** fundamentals, fostering logical thinking and problem solving.
+Developed hands-on STEAM activities and collaborative workshops that increased engagement and practical skills application in young learners.
+Assessed student progress, mentored assistants and iterated course materials to improve learning outcomes and classroom management.</t>
   </si>
   <si>
     <t>Quality Assurance Intern
-Executed manual, descriptive and functional testing following **Agile** and **Kanban** methodologies, documenting defects and validating fixes to improve software reliability.
-Managed issue tracking and test workflows using **Jira**, supporting regression testing, defect triage and release readiness.
-Prepared and maintained **test documentation** and contributed process improvement suggestions that streamlined QA activities and reporting.</t>
-  </si>
-  <si>
-    <t>Automation &amp; PLC Engineering Intern
-Contributed to implementation projects for **AGV** systems, performing design support, assembly, programming and commissioning to integrate automated vehicles into production lines.
-Developed and programmed control logic using **PLC Programming**, conducted start-up, troubleshooting and preventive maintenance of automation equipment.
-Performed system integration and validation testing, produced technical documentation and supported operational handover to maintenance and operations teams.</t>
-  </si>
-  <si>
-    <t>STEM Instructor &amp; Lecturer
-Designed and delivered programming, robotics and electronics curricula for children (4–15) emphasizing **STEAM**, hands-on projects and computational thinking to foster sustained engagement.
-Led university practical sessions for **Electrical Circuits**, developed lab exercises, graded assessments and mentored teaching assistants to improve student learning outcomes.
-Created instructional materials and applied **active-learning methodologies** to increase practical competency and curiosity-driven problem solving.</t>
+Supported QA team in executing **manual testing**, **functional testing** and defect reproduction, producing clear **test documentation** and reproduction steps.
+Worked within **Agile**/**Kanban** frameworks to manage test cycles and track progress using **Jira**, contributing to faster defect resolution and release readiness.
+Collaborated with developers and analysts to validate fixes, prioritize bugs and improve test coverage and quality processes.</t>
+  </si>
+  <si>
+    <t>Engineering Intern — AGV &amp; PLC Projects
+Participated in design and implementation of **AGV** systems, contributing to mechanical layouts, integration plans and operational testing.
+Programmed and commissioned control systems using **PLC Programming**, performing debugging, commissioning and preventive maintenance activities.
+Prepared technical drawings and documentation with **AutoCAD**, supported system bring-up and provided hands-on troubleshooting during deployment.</t>
   </si>
 </sst>
 </file>

</xml_diff>

<commit_message>
clean up data/input files and add an arg in generate_one_pager to save backup csv
</commit_message>
<xml_diff>
--- a/backend/data/output/one_pager_summary.xlsx
+++ b/backend/data/output/one_pager_summary.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="26" uniqueCount="26">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="24" uniqueCount="24">
   <si>
     <t>section_name</t>
   </si>
@@ -25,9 +25,6 @@
     <t>NAME</t>
   </si>
   <si>
-    <t>TOWER</t>
-  </si>
-  <si>
     <t>PROFILE OVERVIEW</t>
   </si>
   <si>
@@ -61,37 +58,32 @@
     <t>Paula María Fernández</t>
   </si>
   <si>
-    <t>Tower 1</t>
-  </si>
-  <si>
-    <t>Electronic engineer and project manager experienced in leading MES and automation initiatives as product owner and coordinating multidisciplinary teams. Skilled in **Python**, **SQL**, **Power BI**, **ETL**, **analytics**, **automation** and PLC programming; strong focus on requirements, delivery and process optimization.</t>
+    <t>Electronic engineer and project manager with experience implementing MES and automation projects, leveraging **Python**, **SQL**, **Power BI**, **ETL** and **data analytics** to enable data-driven decisions and operational automation. Proven product ownership, PLC programming and QA experience delivering IT-manufacturing integrations, process improvements and stakeholder-aligned solutions.</t>
   </si>
   <si>
     <t>Bachelor of Electronic Engineering
-Postgraduate Project Management</t>
+Postgraduate Project Management (PMI Course)</t>
   </si>
   <si>
     <t>Automotive
 Industrial
-High Tech
-Software and Platforms</t>
-  </si>
-  <si>
-    <t>Project Management Lead
-Product Owner MES
-Automation Systems Engineer
-Data Analytics Specialist
-Quality Assurance Analyst
-PLC Programming Engineer</t>
-  </si>
-  <si>
-    <t>Project Management PMI
-Data Analytics
-Python
+Software and Platforms
+High Tech</t>
+  </si>
+  <si>
+    <t>Senior Data Engineer
+IT Project Manager
+MES Product Owner
+Quality Assurance Engineer
+Industrial Automation Engineer</t>
+  </si>
+  <si>
+    <t>Python
 SQL
 Power BI
+Data Analytics
+PMI Project Management
 PLC Programming
-Agile Kanban
 Jira
 MS Project</t>
   </si>
@@ -101,28 +93,28 @@
   </si>
   <si>
     <t>Senior Project Engineering Analyst
-Acted as business product owner for implementation of **MES** projects within **IT**, defining functional requirements and delivering end-user and analyst **training**.
-Managed investment projects for production machinery, overseeing **project management** activities including planning, execution, monitoring and change control.
-Coordinated **multidisciplinary teams**, defined technical specifications and led **vendor management** to ensure on-time delivery of hardware and software components.
-Controlled schedules, resource allocation and budgets using **MS Project**, driving requirements prioritization and alignment with global IT initiatives.</t>
+Served as **Business Product Owner** for MES implementations, defining **functional requirements**, user stories and delivering end-user and executive training to ensure adoption.
+Managed capital equipment projects including planning, execution, budget control and resource allocation using **MS Project** and financial oversight.
+Coordinated multidisciplinary teams and external suppliers, authored technical specifications and integrated solutions with global IT initiatives using **AutoCAD** for technical reviews.
+Defined MES functionalities and led rollout activities to optimize production processes and KPI performance.</t>
   </si>
   <si>
     <t>Senior Programming and Robotics Instructor
-Designed and delivered age-appropriate curricula to teach **programming**, **robotics** and **electronics** fundamentals, fostering logical thinking and problem solving.
-Developed hands-on STEAM activities and collaborative workshops that increased engagement and practical skills application in young learners.
-Assessed student progress, mentored assistants and iterated course materials to improve learning outcomes and classroom management.</t>
-  </si>
-  <si>
-    <t>Quality Assurance Intern
-Supported QA team in executing **manual testing**, **functional testing** and defect reproduction, producing clear **test documentation** and reproduction steps.
-Worked within **Agile**/**Kanban** frameworks to manage test cycles and track progress using **Jira**, contributing to faster defect resolution and release readiness.
-Collaborated with developers and analysts to validate fixes, prioritize bugs and improve test coverage and quality processes.</t>
-  </si>
-  <si>
-    <t>Engineering Intern — AGV &amp; PLC Projects
-Participated in design and implementation of **AGV** systems, contributing to mechanical layouts, integration plans and operational testing.
-Programmed and commissioned control systems using **PLC Programming**, performing debugging, commissioning and preventive maintenance activities.
-Prepared technical drawings and documentation with **AutoCAD**, supported system bring-up and provided hands-on troubleshooting during deployment.</t>
+Designed and delivered age-appropriate curricula focused on **electronics**, **programming** and **STEAM** skills for learners aged 4–15, promoting active and collaborative learning.
+Developed hands-on projects integrating microcontrollers and block/text-based coding to build logical thinking and problem-solving capabilities.
+Mentored assistants, assessed student progress, adapted materials for varied skill levels and fostered curiosity through project-based pedagogy.</t>
+  </si>
+  <si>
+    <t>QA Intern — Quality Assurance
+Supported **Quality Assurance** workflows under **Agile**/**Kanban** methodologies, managing tasks and defects in **Jira** to maintain development cadence.
+Executed manual, descriptive and functional testing, documented test cases and bug reports, and performed regression checks to improve product stability.
+Collaborated with QA and development teams to prioritize fixes, streamline triage processes and support release readiness.</t>
+  </si>
+  <si>
+    <t>Automation Engineering Intern — AGV &amp; PLC Projects
+Contributed to design, assembly, programming and commissioning of **AGV** systems, performing integration tests and operational validation.
+Developed and debugged **PLC** programs, conducted start-up procedures, troubleshooting and preventive maintenance to ensure reliable automation.
+Prepared technical documentation, test reports and collaborated with cross-functional teams to deploy safe, efficient automated solutions.</t>
   </si>
 </sst>
 </file>
@@ -480,7 +472,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:B13"/>
+  <dimension ref="A1:B12"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:2">
@@ -496,7 +488,7 @@
         <v>2</v>
       </c>
       <c r="B2" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
     </row>
     <row r="3" spans="1:2">
@@ -504,7 +496,7 @@
         <v>3</v>
       </c>
       <c r="B3" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
     </row>
     <row r="4" spans="1:2">
@@ -512,7 +504,7 @@
         <v>4</v>
       </c>
       <c r="B4" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
     </row>
     <row r="5" spans="1:2">
@@ -520,7 +512,7 @@
         <v>5</v>
       </c>
       <c r="B5" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
     </row>
     <row r="6" spans="1:2">
@@ -528,7 +520,7 @@
         <v>6</v>
       </c>
       <c r="B6" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
     </row>
     <row r="7" spans="1:2">
@@ -536,7 +528,7 @@
         <v>7</v>
       </c>
       <c r="B7" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
     </row>
     <row r="8" spans="1:2">
@@ -544,7 +536,7 @@
         <v>8</v>
       </c>
       <c r="B8" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
     </row>
     <row r="9" spans="1:2">
@@ -552,7 +544,7 @@
         <v>9</v>
       </c>
       <c r="B9" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
     </row>
     <row r="10" spans="1:2">
@@ -560,7 +552,7 @@
         <v>10</v>
       </c>
       <c r="B10" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
     </row>
     <row r="11" spans="1:2">
@@ -568,7 +560,7 @@
         <v>11</v>
       </c>
       <c r="B11" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
     </row>
     <row r="12" spans="1:2">
@@ -576,15 +568,7 @@
         <v>12</v>
       </c>
       <c r="B12" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="13" spans="1:2">
-      <c r="A13" t="s">
-        <v>13</v>
-      </c>
-      <c r="B13" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Deleted personal pdfs file and added function to clean up any personal data after use
</commit_message>
<xml_diff>
--- a/backend/data/output/one_pager_summary.xlsx
+++ b/backend/data/output/one_pager_summary.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="25" uniqueCount="25">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="26" uniqueCount="26">
   <si>
     <t>section_name</t>
   </si>
@@ -58,13 +58,16 @@
     <t>Role_4</t>
   </si>
   <si>
+    <t>LEANDRO FASSA</t>
+  </si>
+  <si>
     <t>CONTROL TOWER</t>
   </si>
   <si>
-    <t>Experienced data engineer focused on building scalable data platforms and analytics solutions, with expertise in **data engineering**, **ETL**, **data quality**, and **data warehousing**. Hands-on with **AWS**, **Snowflake**, **SQL**, **Python**, **Airflow**, **Matillion**, and delivering **Power BI** reporting and SAP PP/MM support for supply chain.</t>
-  </si>
-  <si>
-    <t>Bachelor Degree in Industrial Engineering</t>
+    <t>Experienced data engineer with strong background in **data engineering**, **ETL**, **SQL** and **Python**, leveraging cloud platforms and warehouses (AWS, Snowflake) to build reliable pipelines. Proven in **data quality** remediation, pipeline orchestration and **analytics** reporting using **Power BI** to support supply chain and financial stakeholders.</t>
+  </si>
+  <si>
+    <t>Bachelor of Industrial Engineering</t>
   </si>
   <si>
     <t>Banking
@@ -74,20 +77,21 @@
   </si>
   <si>
     <t>Senior Data Engineer
-Data Warehouse Analyst
-Platform Software Engineer
+Senior Data Analyst
+Software Engineer Platform
 Supply Chain Analyst
 SAP Consultant PP/MM</t>
   </si>
   <si>
     <t>AWS Cloud Practitioner
-Microsoft Power BI
+Power BI
 SQL
 Python
 Snowflake
 Microsoft SSIS
+Airflow
 Matillion
-Airflow
+Big Data Quality Management
 Azure DP-900</t>
   </si>
   <si>
@@ -95,28 +99,28 @@
 English C1</t>
   </si>
   <si>
-    <t>Software Engineer Platform – Software platforms
-Designed and implemented scalable data models and services on **SAP BTP** using the **CAP** framework to enable structured backend APIs for enterprise applications.
-Developed and maintained backend data services that enforce business logic and ensure **data integrity**, supporting analytics and reporting pipelines.
-Collaborated with platform teams to integrate services with analytics consumers and improve service reliability and observability.</t>
-  </si>
-  <si>
-    <t>Data Engineer, Quality – Financial Services
-Investigated and resolved data quality issues across the **AWS** data lake, performing root cause analysis with **S3**, **Athena**, **EMR**, **DynamoDB**, and **CloudWatch**.
-Implemented and improved integrity rules in **OvalEdge** using **SQL**, reducing recurring data incidents and impacting ~10% of reported issues.
-Produced **Power BI** reports to communicate quality findings and mentored new team members on data workflows and quality controls.</t>
-  </si>
-  <si>
-    <t>Data Engineer – Financial Services
-Built an end-to-end ingestion pipeline from **Qualtrics** into the **AWS** data lake and loaded curated datasets into **Snowflake** using **Python**, **SQL**, and **GitLab**, orchestrated with **Airflow**.
-Transformed raw data into analytics-ready tables in **Snowflake**, resolving ~40% of data quality issues and improving downstream reporting accuracy.
-Developed an **ELT** process in **Matillion** to support Customer Experience stakeholders, optimizing data delivery and traceability.</t>
-  </si>
-  <si>
-    <t>Data Warehouse Analyst – Oil &amp; Gas
-Monitored and analyzed ETL workflows in **SSIS**, performing **SQL** performance analysis to identify pipeline bottlenecks, anomalies, and inefficiencies.
-Delivered a **Power BI** report on data warehouse performance that uncovered optimization opportunities and reduced failures due to package dependencies by 15%.
-Executed data troubleshooting and remediation to improve ETL reliability and support operational analytics.</t>
+    <t>Software Engineer Platform
+Design and implement data models on **SAP BTP** using the **CAP framework** to enable structured backend data services for enterprise applications.
+Develop and maintain backend services that enforce business logic and **data integrity**, supporting analytics and reporting consumers.
+Integrate platform components with **Snowflake**, **SQL**, and ETL tools to optimize data access, performance, and service reliability.</t>
+  </si>
+  <si>
+    <t>Data Engineer, Quality
+Resolved **data quality** incidents in the AWS data lake through root-cause analysis using **S3**, **Athena**, **EMR**, **DynamoDB**, **CloudWatch**, and **Snowflake**.
+Enhanced integrity rules in **OvalEdge** with **SQL**, reducing ~10% of recurring issues and produced **Power BI** reports to drive remediation and stakeholder visibility.
+Mentored new hires on data workflows, tooling, and quality processes to accelerate onboarding and sustain operational standards.</t>
+  </si>
+  <si>
+    <t>Data Engineer
+Built end-to-end ingestion pipelines from **Qualtrics** into the AWS data lake (**S3**, **Athena**, **EMR**, **DynamoDB**) and loaded analytics-ready datasets into **Snowflake** using **Python**, **SQL**, and **GitLab**.
+Orchestrated workflows with **Airflow** and developed ELT processes in **Matillion**, resolving ~40% of data quality issues and enabling Customer Experience analytics.
+Transformed raw sources into optimized Snowflake schemas to improve downstream reporting performance and data reliability.</t>
+  </si>
+  <si>
+    <t>Supply Chain Analyst
+Analyzed inventory and production datasets using **SAP PP/MM** and advanced **Excel** to support supply chain planning and KPI tracking.
+Collaborated with Production and Sales to deliver interactive operational dashboards and reports using **Power BI** and Excel visualizations for faster decision-making.
+Integrated transactional data sources and standardized reporting to improve visibility into inventory levels, production throughput, and planning accuracy.</t>
   </si>
 </sst>
 </file>
@@ -489,13 +493,16 @@
       <c r="A2" t="s">
         <v>2</v>
       </c>
+      <c r="B2" t="s">
+        <v>14</v>
+      </c>
     </row>
     <row r="3" spans="1:2">
       <c r="A3" t="s">
         <v>3</v>
       </c>
       <c r="B3" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
     </row>
     <row r="4" spans="1:2">
@@ -503,7 +510,7 @@
         <v>4</v>
       </c>
       <c r="B4" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
     </row>
     <row r="5" spans="1:2">
@@ -511,7 +518,7 @@
         <v>5</v>
       </c>
       <c r="B5" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
     </row>
     <row r="6" spans="1:2">
@@ -519,7 +526,7 @@
         <v>6</v>
       </c>
       <c r="B6" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
     </row>
     <row r="7" spans="1:2">
@@ -527,7 +534,7 @@
         <v>7</v>
       </c>
       <c r="B7" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
     </row>
     <row r="8" spans="1:2">
@@ -535,7 +542,7 @@
         <v>8</v>
       </c>
       <c r="B8" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
     </row>
     <row r="9" spans="1:2">
@@ -543,7 +550,7 @@
         <v>9</v>
       </c>
       <c r="B9" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
     </row>
     <row r="10" spans="1:2">
@@ -551,7 +558,7 @@
         <v>10</v>
       </c>
       <c r="B10" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
     </row>
     <row r="11" spans="1:2">
@@ -559,7 +566,7 @@
         <v>11</v>
       </c>
       <c r="B11" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
     </row>
     <row r="12" spans="1:2">
@@ -567,7 +574,7 @@
         <v>12</v>
       </c>
       <c r="B12" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
     </row>
     <row r="13" spans="1:2">
@@ -575,7 +582,7 @@
         <v>13</v>
       </c>
       <c r="B13" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
     </row>
   </sheetData>

</xml_diff>